<commit_message>
fixx: export to xlsx torque & angle
</commit_message>
<xml_diff>
--- a/docs/Worksheet in Software%20development%20-%20R2.xlsx
+++ b/docs/Worksheet in Software%20development%20-%20R2.xlsx
@@ -156,8 +156,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TorqueSummary" displayName="TorqueSummary" ref="A1:L4" headerRowCount="1">
-  <autoFilter ref="A1:L4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TorqueSummary" displayName="TorqueSummary" ref="A1:L7" headerRowCount="1">
+  <autoFilter ref="A1:L7"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Line No"/>
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" style="1" min="1" max="4"/>
@@ -687,7 +687,6 @@
           <t>Inner Tie Rod</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Breakaway Torque</t>
@@ -722,6 +721,146 @@
           <t>DS2B3DS</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ITR #1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I5" t="n">
+        <v>30</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3.627381</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ITR #1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I6" t="n">
+        <v>30</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3.627381</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ITR #1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I7" t="n">
+        <v>30</v>
+      </c>
+      <c r="J7" t="n">
+        <v>3.627381</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update: documentation worksheet and plc project file
</commit_message>
<xml_diff>
--- a/docs/Worksheet in Software%20development%20-%20R2.xlsx
+++ b/docs/Worksheet in Software%20development%20-%20R2.xlsx
@@ -156,8 +156,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TorqueSummary" displayName="TorqueSummary" ref="A1:L7" headerRowCount="1">
-  <autoFilter ref="A1:L7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TorqueSummary" displayName="TorqueSummary" ref="A1:L13" headerRowCount="1">
+  <autoFilter ref="A1:L13"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Line No"/>
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" style="1" min="1" max="4"/>
@@ -830,7 +830,6 @@
           <t>Inner Tie Rod</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Breakaway Torque</t>
@@ -860,7 +859,266 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ITR #1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I8" t="n">
+        <v>30</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ITR #1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I9" t="n">
+        <v>30</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ITR #1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ITR #1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I11" t="n">
+        <v>30</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ITR #1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>-30</v>
+      </c>
+      <c r="I12" t="n">
+        <v>30</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>S/Link #1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>-29.999996</v>
+      </c>
+      <c r="I13" t="n">
+        <v>30</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>